<commit_message>
feat: add interactive product showcase, comparison section, and landing page components
</commit_message>
<xml_diff>
--- a/Bang_Du_Toan_Chi_Phi.xlsx
+++ b/Bang_Du_Toan_Chi_Phi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\OJT-Review\nguyetnhan_phohien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5501083E-24DE-46E6-A1FA-B04D35C5E811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0237929-75EE-44EF-9EA9-70DBF2E7E1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,12 +127,6 @@
     <t>Cơ sở dữ liệu (PostgreSQL)</t>
   </si>
   <si>
-    <t>Supabase</t>
-  </si>
-  <si>
-    <t>Free Plan (500MB Database, 5GB Egress, Shared CPU)</t>
-  </si>
-  <si>
     <t>Miễn phí 500MB DB (lưu được hàng chục nghìn đơn hàng &amp; sản phẩm). Có giao diện quản lý bảng trực quan.</t>
   </si>
   <si>
@@ -187,9 +181,6 @@
     <t>Tên miền (nguyetnhanphohien.com)</t>
   </si>
   <si>
-    <t>Hạ tầng (Railway $5 + GCS $0.5)</t>
-  </si>
-  <si>
     <t>Bảo mật SSL + Vercel + Supabase + Email</t>
   </si>
   <si>
@@ -197,6 +188,15 @@
   </si>
   <si>
     <t>★ TỔNG CHI PHÍ</t>
+  </si>
+  <si>
+    <t>Hạ tầng (Railway $5 + GCS $5)</t>
+  </si>
+  <si>
+    <t>Plan (32G Database, 5GB Egress, Shared CPU)</t>
+  </si>
+  <si>
+    <t>Azure SQL</t>
   </si>
 </sst>
 </file>
@@ -208,7 +208,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0\ &quot;₫&quot;"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,6 +261,14 @@
       <sz val="11"/>
       <color rgb="FF047857"/>
       <name val="Segoe UI"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -361,10 +369,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -408,42 +417,44 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -457,6 +468,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>579540</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>113416</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FA74005-DE6F-DA96-BD96-8DB8B3388ECA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16163365" y="2510118"/>
+          <a:ext cx="4846740" cy="5303980"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -744,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -757,31 +823,31 @@
     <col min="8" max="8" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.3">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+    </row>
+    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.3">
       <c r="F3" s="1" t="s">
         <v>2</v>
       </c>
@@ -789,7 +855,7 @@
         <v>25500</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -815,19 +881,19 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-    </row>
-    <row r="7" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+    </row>
+    <row r="7" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -854,7 +920,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>2</v>
       </c>
@@ -879,8 +945,9 @@
       <c r="H8" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="35"/>
+    </row>
+    <row r="9" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
         <v>22</v>
       </c>
@@ -899,20 +966,21 @@
       <c r="H9" s="10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="24" t="s">
+      <c r="K9" s="35"/>
+    </row>
+    <row r="10" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-    </row>
-    <row r="11" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+    </row>
+    <row r="11" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>3</v>
       </c>
@@ -938,7 +1006,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>4</v>
       </c>
@@ -965,7 +1033,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>5</v>
       </c>
@@ -973,54 +1041,54 @@
         <v>34</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>28</v>
       </c>
       <c r="F13" s="6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G13" s="7">
-        <v>0</v>
+        <v>255000</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>6</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>28</v>
       </c>
       <c r="F14" s="6">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="G14" s="7">
         <f>F14*$G$3</f>
-        <v>140250</v>
+        <v>127500</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -1028,40 +1096,40 @@
       <c r="E15" s="20"/>
       <c r="F15" s="8">
         <f>SUM(F11:F14)</f>
-        <v>10.5</v>
+        <v>20</v>
       </c>
       <c r="G15" s="9">
         <f>SUM(G11:G14)</f>
-        <v>267750</v>
+        <v>510000</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>7</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>28</v>
@@ -1073,12 +1141,12 @@
         <v>0</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="20"/>
@@ -1093,33 +1161,33 @@
         <v>0</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
+      <c r="A19" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
       <c r="F19" s="11">
         <f>F15+F18</f>
-        <v>10.5</v>
+        <v>20</v>
       </c>
       <c r="G19" s="12">
         <f>G15+G18</f>
-        <v>267750</v>
+        <v>510000</v>
       </c>
       <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="31"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="16"/>
@@ -1135,91 +1203,101 @@
       <c r="H21" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+    </row>
+    <row r="24" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-    </row>
-    <row r="24" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="18"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="23"/>
     </row>
     <row r="25" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
+      <c r="A25" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
       <c r="D25" s="7">
         <v>248000</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="18"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="23"/>
     </row>
     <row r="26" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
+      <c r="A26" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
       <c r="D26" s="7">
         <f>G19</f>
-        <v>267750</v>
+        <v>510000</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="18"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="23"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
+      <c r="A27" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
       <c r="D27" s="7">
         <v>0</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="18"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="23"/>
     </row>
     <row r="28" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
+      <c r="A28" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
       <c r="D28" s="15">
         <f>SUM(D25:D27)</f>
-        <v>515750</v>
+        <v>758000</v>
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="26"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A21:E21"/>
@@ -1232,17 +1310,8 @@
     <mergeCell ref="G25:H25"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add product showcase components, interactive sections, and landing page views
</commit_message>
<xml_diff>
--- a/Bang_Du_Toan_Chi_Phi.xlsx
+++ b/Bang_Du_Toan_Chi_Phi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\OJT-Review\nguyetnhan_phohien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0237929-75EE-44EF-9EA9-70DBF2E7E1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6A33E4-B50F-4E38-9D43-FDB4B7D10689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -417,33 +417,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -451,7 +433,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -824,28 +824,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.35">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.3">
       <c r="F3" s="1" t="s">
@@ -882,16 +882,16 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
@@ -945,16 +945,16 @@
       <c r="H8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="35"/>
+      <c r="K8" s="17"/>
     </row>
     <row r="9" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
       <c r="F9" s="8">
         <f>SUM(F7:F8)</f>
         <v>9.7254901960784306</v>
@@ -966,19 +966,19 @@
       <c r="H9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="35"/>
+      <c r="K9" s="17"/>
     </row>
     <row r="10" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
@@ -1023,11 +1023,11 @@
         <v>28</v>
       </c>
       <c r="F12" s="6">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G12" s="7">
         <f>F12*$G$3</f>
-        <v>127500</v>
+        <v>510000</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>33</v>
@@ -1087,36 +1087,36 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="8">
         <f>SUM(F11:F14)</f>
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G15" s="9">
         <f>SUM(G11:G14)</f>
-        <v>510000</v>
+        <v>892500</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
@@ -1145,13 +1145,13 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
       <c r="F18" s="8">
         <f>F17</f>
         <v>0</v>
@@ -1165,139 +1165,129 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
       <c r="F19" s="11">
         <f>F15+F18</f>
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G19" s="12">
         <f>G15+G18</f>
-        <v>510000</v>
+        <v>892500</v>
       </c>
       <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="A20" s="32"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
       <c r="F20" s="14"/>
       <c r="G20" s="15"/>
       <c r="H20" s="16"/>
     </row>
     <row r="21" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="8"/>
       <c r="G21" s="9"/>
       <c r="H21" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
     </row>
     <row r="24" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="3" t="s">
         <v>51</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="23"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="21"/>
     </row>
     <row r="25" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="7">
         <v>248000</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="23"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="21"/>
     </row>
     <row r="26" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="7">
         <f>G19</f>
-        <v>510000</v>
+        <v>892500</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="23"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="7">
         <v>0</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="23"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="21"/>
     </row>
     <row r="28" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
       <c r="D28" s="15">
         <f>SUM(D25:D27)</f>
-        <v>758000</v>
+        <v>1140500</v>
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="18"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A9:E9"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A21:E21"/>
@@ -1310,6 +1300,16 @@
     <mergeCell ref="G25:H25"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>